<commit_message>
Removed 2nd sentence in Description.  Updated negative test case 2 with ae.xpt.
</commit_message>
<xml_diff>
--- a/rules/CORE-000172/negative/02/data/unit-test-coreid-CG0409-negative-2.xlsx
+++ b/rules/CORE-000172/negative/02/data/unit-test-coreid-CG0409-negative-2.xlsx
@@ -38,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -55,7 +55,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -66,12 +65,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -79,12 +74,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -120,15 +109,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,10 +459,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -487,7 +475,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -498,24 +486,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Subject Elements</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Demographics</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>Adverse Events</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -545,82 +541,82 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>$dm_studyid</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>5</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E4" s="4" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="F4" s="4" t="str">
         <v>CDISCPILOT02</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="4">
         <v>5</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>$dm_studyid</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
     </row>
@@ -671,22 +667,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="5" t="str">
         <v>Element Code</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="5" t="str">
         <v>Description of Element</v>
       </c>
       <c r="G2" s="5" t="str">
@@ -776,142 +772,142 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>SCREEN</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>Screening</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>2012-11-23</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="4">
         <v>-7</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>LOWER</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>Zanomaline 54 mg</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="4" t="str">
         <v>2013-05-20</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="4">
         <v>1</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="4">
         <v>172</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="str">
+      <c r="A7" s="6" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>1</v>
       </c>
-      <c r="E7" s="6" t="str">
+      <c r="E7" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F7" s="4" t="str">
         <v>Screening</v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G7" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H7" s="4" t="str">
         <v>2012-10-30</v>
       </c>
-      <c r="I7" s="6" t="str">
+      <c r="I7" s="4" t="str">
         <v>2012-11-15</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="4">
         <v>-16</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
-      <c r="B8" s="6" t="str">
+      <c r="B8" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>2</v>
       </c>
-      <c r="E8" s="6" t="str">
+      <c r="E8" s="4" t="str">
         <v>HIGHEST</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="4" t="str">
         <v>Zanomaline 54 mg</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="4" t="str">
         <v>2012-11-15</v>
       </c>
-      <c r="I8" s="6" t="str">
+      <c r="I8" s="4" t="str">
         <v>2013-01-14</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="4">
         <v>1</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="4">
         <v>61</v>
       </c>
     </row>
@@ -1247,82 +1243,82 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="4" t="str">
         <v>1115</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>2013-01-23</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>2013-01-23</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>2012-11-23</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="4" t="str">
         <v>2013-05-20</v>
       </c>
-      <c r="K5" s="2" t="str">
+      <c r="K5" s="4" t="str">
         <v/>
       </c>
-      <c r="L5" s="2" t="str">
+      <c r="L5" s="4" t="str">
         <v/>
       </c>
-      <c r="M5" s="6" t="str">
+      <c r="M5" s="4" t="str">
         <v>701</v>
       </c>
-      <c r="N5" s="6" t="str">
+      <c r="N5" s="4" t="str">
         <v>1928</v>
       </c>
-      <c r="O5" s="6">
+      <c r="O5" s="4">
         <v>84</v>
       </c>
-      <c r="P5" s="6" t="str">
+      <c r="P5" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q5" s="6" t="str">
+      <c r="Q5" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="R5" s="6" t="str">
+      <c r="R5" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S5" s="6" t="str">
+      <c r="S5" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T5" s="6" t="str">
+      <c r="T5" s="4" t="str">
         <v>ZAN_LOW</v>
       </c>
-      <c r="U5" s="6" t="str">
+      <c r="U5" s="4" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
-      <c r="V5" s="6" t="str">
+      <c r="V5" s="4" t="str">
         <v>ZAN_LOW</v>
       </c>
-      <c r="W5" s="6" t="str">
+      <c r="W5" s="4" t="str">
         <v>Zanomaline Low Dose (54 mg)</v>
       </c>
-      <c r="X5" s="2" t="str">
+      <c r="X5" s="4" t="str">
         <v/>
       </c>
-      <c r="Y5" s="2" t="str">
+      <c r="Y5" s="4" t="str">
         <v/>
       </c>
-      <c r="Z5" s="6" t="str">
+      <c r="Z5" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
@@ -1658,236 +1654,236 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="str">
+      <c r="A5" s="6" t="str">
         <v>CDISCPILOT02</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>AE</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>2</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>FATIGUE</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>MODERATE</v>
       </c>
-      <c r="G5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="H5" s="6" t="str">
+      <c r="G5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="H5" s="4" t="str">
         <v>DOSE NOT CHANGED</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>UNLIKELY RELATED</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="4" t="str">
         <v>NOT RECOVERED/NOT RESOLVED</v>
       </c>
-      <c r="K5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="L5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="M5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="N5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="O5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="P5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="Q5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="R5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="S5" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="T5" s="6" t="str">
+      <c r="K5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="L5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="M5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="N5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="O5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="P5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="Q5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="R5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="S5" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="T5" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="U5" s="6" t="str">
+      <c r="U5" s="4" t="str">
         <v>2013-01-14</v>
       </c>
-      <c r="V5" s="2" t="str">
+      <c r="V5" s="4" t="str">
         <v/>
       </c>
-      <c r="W5" s="6">
+      <c r="W5" s="4">
         <v>46</v>
       </c>
-      <c r="X5" s="2" t="str">
+      <c r="X5" s="4" t="str">
         <v/>
       </c>
-      <c r="Y5" s="6" t="str">
+      <c r="Y5" s="4" t="str">
         <v>ONGOING</v>
       </c>
-      <c r="Z5" s="6" t="str">
+      <c r="Z5" s="4" t="str">
         <v>2013-05-20</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
         <v>AE</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>1</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>HYPERHIDROSIS</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>MILD</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <v>DOSE NOT CHANGED</v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="4" t="str">
         <v>POSSIBLY RELATED</v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="4" t="str">
         <v>NOT RECOVERED/NOT RESOLVED</v>
       </c>
-      <c r="K6" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="L6" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="M6" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="N6" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="O6" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="P6" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="Q6" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="R6" s="6" t="str">
+      <c r="K6" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="L6" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="M6" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="N6" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="O6" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="P6" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="Q6" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="R6" s="4" t="str">
         <v/>
       </c>
-      <c r="S6" s="6" t="str">
+      <c r="S6" s="4" t="str">
         <v/>
       </c>
-      <c r="T6" s="6" t="str">
+      <c r="T6" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="U6" s="6" t="str">
+      <c r="U6" s="4" t="str">
         <v>2013-08-30</v>
       </c>
-      <c r="V6" s="2" t="str">
+      <c r="V6" s="4" t="str">
         <v/>
       </c>
-      <c r="W6" s="6">
+      <c r="W6" s="4">
         <v>2</v>
       </c>
-      <c r="X6" s="2" t="str">
+      <c r="X6" s="4" t="str">
         <v/>
       </c>
-      <c r="Y6" s="6" t="str">
+      <c r="Y6" s="4" t="str">
         <v>ONGOING</v>
       </c>
-      <c r="Z6" s="6" t="str">
+      <c r="Z6" s="4" t="str">
         <v>2013-02-13</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT1</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="4" t="str">
         <v>AE</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC008</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>1</v>
       </c>
-      <c r="E7" s="6" t="str">
+      <c r="E7" s="4" t="str">
         <v>COMPLETED SUICIDE</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F7" s="4" t="str">
         <v>SEVERE</v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G7" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H7" s="4" t="str">
         <v>DRUG WITHDRAWN</v>
       </c>
-      <c r="I7" s="6" t="str">
+      <c r="I7" s="4" t="str">
         <v>NOT RELATED</v>
       </c>
-      <c r="J7" s="6" t="str">
+      <c r="J7" s="4" t="str">
         <v>FATAL</v>
       </c>
-      <c r="K7" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="L7" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="M7" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="N7" s="6" t="str">
+      <c r="K7" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="L7" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="M7" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="N7" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="O7" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="P7" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="Q7" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="R7" s="6" t="str">
-        <v>N</v>
-      </c>
-      <c r="S7" s="6" t="str">
+      <c r="O7" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="P7" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="Q7" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="R7" s="4" t="str">
+        <v>N</v>
+      </c>
+      <c r="S7" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="T7" s="6" t="str">
+      <c r="T7" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="U7" s="6" t="str">
+      <c r="U7" s="4" t="str">
         <v>2014-10-31</v>
       </c>
-      <c r="V7" s="6" t="str">
+      <c r="V7" s="4" t="str">
         <v>2014-10-31</v>
       </c>
-      <c r="W7" s="6">
+      <c r="W7" s="4">
         <v>174</v>
       </c>
-      <c r="X7" s="6">
+      <c r="X7" s="4">
         <v>174</v>
       </c>
     </row>

</xml_diff>